<commit_message>
docs: actualizar la hoja de Excel de pruebas unitarias
Versión guardada desde Excel de docs/pruebas_unitarias.xlsx: 41 casos con la columna Estado en español (Pasa/Falla) y sin colores.
</commit_message>
<xml_diff>
--- a/docs/pruebas_unitarias.xlsx
+++ b/docs/pruebas_unitarias.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\Downloads\99 - OTROS\calculator-v1.1.0\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\Downloads\99 - OTROS\calculator-v1.1.0\TRABAJO-DE-CALIDAD-DE-SOFTWARE\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9D2ECA5-6BF2-4A0B-8191-3A3654EB1BBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4FAF4B6-D334-4066-9C2A-742A2C96DF35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -579,22 +579,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -858,10 +843,10 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="51.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="50.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16.5546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="46" customWidth="1"/>
+    <col min="4" max="4" width="17.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="40.6640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="10" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1028,7 +1013,7 @@
         <v>-5</v>
       </c>
       <c r="G7" s="5" t="str">
-        <f t="shared" ref="G2:G42" si="0">IF(E7=F7,"Pasa","Falla")</f>
+        <f t="shared" ref="G7:G39" si="0">IF(E7=F7,"Pasa","Falla")</f>
         <v>Pasa</v>
       </c>
     </row>

</xml_diff>